<commit_message>
HEP_concordances: 8 university name variants (user); rerun ORCID bulk pass
Kept ACIFs with an ORCID 16,518 -> 16,525; ACIFs 23,288 -> 23,285.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_persisted/HEP_concordances.xlsx
+++ b/data_persisted/HEP_concordances.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Variants" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="224">
   <si>
     <t xml:space="preserve">Variants</t>
   </si>
@@ -102,6 +102,9 @@
     <t xml:space="preserve">La Trobe University</t>
   </si>
   <si>
+    <t xml:space="preserve">Latrobe University</t>
+  </si>
+  <si>
     <t xml:space="preserve">Macquarie University</t>
   </si>
   <si>
@@ -120,6 +123,9 @@
     <t xml:space="preserve">Royal Melbourne Institute of Technology University</t>
   </si>
   <si>
+    <t xml:space="preserve">Royal Melbourne Institute of Technology</t>
+  </si>
+  <si>
     <t xml:space="preserve">Southern Cross University</t>
   </si>
   <si>
@@ -135,6 +141,9 @@
     <t xml:space="preserve">University of Adelaide</t>
   </si>
   <si>
+    <t xml:space="preserve">Adelaide University</t>
+  </si>
+  <si>
     <t xml:space="preserve">University of Canberra</t>
   </si>
   <si>
@@ -162,6 +171,15 @@
     <t xml:space="preserve">UNSW Sydney</t>
   </si>
   <si>
+    <t xml:space="preserve">UNSW Australia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNSW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of New South Wales Sydney</t>
+  </si>
+  <si>
     <t xml:space="preserve">The University of Newcastle</t>
   </si>
   <si>
@@ -180,6 +198,9 @@
     <t xml:space="preserve">University of Queensland</t>
   </si>
   <si>
+    <t xml:space="preserve">The Univeristy of Queensland</t>
+  </si>
+  <si>
     <t xml:space="preserve">University of South Australia</t>
   </si>
   <si>
@@ -202,6 +223,9 @@
   </si>
   <si>
     <t xml:space="preserve">University of the Sunshine Coast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USC - University of the Sunshine Coast</t>
   </si>
   <si>
     <t xml:space="preserve">The University of Western Australia</t>
@@ -751,7 +775,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -762,6 +786,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -887,8 +915,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B74"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="42.75"/>
   </cols>
@@ -1094,11 +1122,11 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>26</v>
+      <c r="B26" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1138,7 +1166,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1146,15 +1174,15 @@
         <v>32</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>33</v>
+      <c r="B33" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1170,7 +1198,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1186,7 +1214,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1202,7 +1230,7 @@
         <v>39</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1218,7 +1246,7 @@
         <v>41</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1226,7 +1254,7 @@
         <v>42</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1234,7 +1262,7 @@
         <v>43</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1242,7 +1270,7 @@
         <v>44</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1250,7 +1278,7 @@
         <v>45</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1274,7 +1302,7 @@
         <v>48</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1282,23 +1310,23 @@
         <v>49</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>51</v>
+      <c r="B51" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1306,7 +1334,7 @@
         <v>52</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1338,7 +1366,7 @@
         <v>56</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1350,10 +1378,10 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="1" t="s">
+      <c r="A58" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" s="3" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1370,7 +1398,7 @@
         <v>60</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1378,7 +1406,7 @@
         <v>61</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1405,20 +1433,84 @@
         <v>64</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1438,7 +1530,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H43"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.12"/>
@@ -1455,25 +1547,25 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1484,19 +1576,19 @@
         <v>1991</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>2</v>
@@ -1510,19 +1602,19 @@
         <v>1946</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>3</v>
@@ -1536,19 +1628,19 @@
         <v>1990</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>76</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>7</v>
@@ -1562,19 +1654,19 @@
         <v>1989</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>8</v>
@@ -1588,19 +1680,19 @@
         <v>1992</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>9</v>
@@ -1614,19 +1706,19 @@
         <v>2004</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>11</v>
@@ -1640,19 +1732,19 @@
         <v>1989</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>92</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>12</v>
@@ -1666,19 +1758,19 @@
         <v>1987</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H9" s="1" t="s">
         <v>13</v>
@@ -1692,19 +1784,19 @@
         <v>1974</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>15</v>
@@ -1718,19 +1810,19 @@
         <v>1991</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>16</v>
@@ -1744,19 +1836,19 @@
         <v>2014</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>17</v>
@@ -1770,19 +1862,19 @@
         <v>1966</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H13" s="1" t="s">
         <v>19</v>
@@ -1796,19 +1888,19 @@
         <v>1971</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>21</v>
@@ -1822,19 +1914,19 @@
         <v>1970</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>23</v>
@@ -1848,19 +1940,19 @@
         <v>1964</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>25</v>
@@ -1868,704 +1960,704 @@
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1964</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>1958</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>1973</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1989</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>1992</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>1994</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1992</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2014</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>1874</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>1990</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1853</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>1954</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1949</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>1965</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1990</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1909</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1991</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1992</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>1850</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1890</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>1988</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1996</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1911</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>1975</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>1992</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>1989</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -2585,7 +2677,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.03"/>
@@ -2597,22 +2689,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2620,16 +2712,16 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>2</v>
@@ -2640,16 +2732,16 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -2660,16 +2752,16 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>8</v>
@@ -2680,16 +2772,16 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>9</v>
@@ -2700,16 +2792,16 @@
         <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>11</v>
@@ -2720,16 +2812,16 @@
         <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>12</v>
@@ -2740,16 +2832,16 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>13</v>
@@ -2760,16 +2852,16 @@
         <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>15</v>
@@ -2780,16 +2872,16 @@
         <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>16</v>
@@ -2800,16 +2892,16 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>17</v>
@@ -2820,16 +2912,16 @@
         <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>21</v>
@@ -2840,16 +2932,16 @@
         <v>23</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>23</v>
@@ -2860,16 +2952,16 @@
         <v>25</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>25</v>
@@ -2877,142 +2969,142 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3020,16 +3112,16 @@
         <v>4</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>3</v>
@@ -3040,16 +3132,16 @@
         <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>19</v>
@@ -3057,402 +3149,402 @@
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>